<commit_message>
chore(data): refresh works seed via rebuild
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/works.xlsx
+++ b/data/works.xlsx
@@ -707,7 +707,7 @@
         <v>70</v>
       </c>
       <c r="O2" s="2" t="n">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">

</xml_diff>